<commit_message>
Remove linha de fórmula do modelo de Liberação (evita #VALOR!)
Saldo Total e Comissão 6% são calculados pelo sistema e não são lidos
na importação; o modelo passa a conter apenas o cabeçalho.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template_liberacao.xlsx
+++ b/public/template_liberacao.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -502,16 +502,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="H2">
-        <f>F2+G2</f>
-        <v/>
-      </c>
-      <c r="I2">
-        <f>H2*6%</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>